<commit_message>
Complete forensic audit model repair test suite and final deliverables
</commit_message>
<xml_diff>
--- a/outputs/valuation.xlsx
+++ b/outputs/valuation.xlsx
@@ -500,10 +500,10 @@
         <v>3730619</v>
       </c>
       <c r="J2">
-        <v>10756803</v>
+        <v>407884077</v>
       </c>
       <c r="K2">
-        <v>34681.49</v>
+        <v>914.63</v>
       </c>
       <c r="L2" t="s">
         <v>13</v>
@@ -538,10 +538,10 @@
         <v>2431688</v>
       </c>
       <c r="J3">
-        <v>10756803</v>
+        <v>407884077</v>
       </c>
       <c r="K3">
-        <v>22606.04</v>
+        <v>596.17</v>
       </c>
       <c r="L3" t="s">
         <v>14</v>
@@ -576,10 +576,10 @@
         <v>1465095</v>
       </c>
       <c r="J4">
-        <v>10756803</v>
+        <v>407884077</v>
       </c>
       <c r="K4">
-        <v>13620.17</v>
+        <v>359.19</v>
       </c>
       <c r="L4" t="s">
         <v>15</v>
@@ -614,10 +614,10 @@
         <v>1074236</v>
       </c>
       <c r="J5">
-        <v>20895032</v>
+        <v>209000000</v>
       </c>
       <c r="K5">
-        <v>5141.11</v>
+        <v>513.99</v>
       </c>
       <c r="L5" t="s">
         <v>13</v>
@@ -652,10 +652,10 @@
         <v>934697</v>
       </c>
       <c r="J6">
-        <v>20895032</v>
+        <v>209000000</v>
       </c>
       <c r="K6">
-        <v>4473.3</v>
+        <v>447.22</v>
       </c>
       <c r="L6" t="s">
         <v>14</v>
@@ -690,10 +690,10 @@
         <v>637231</v>
       </c>
       <c r="J7">
-        <v>20895032</v>
+        <v>209000000</v>
       </c>
       <c r="K7">
-        <v>3049.68</v>
+        <v>304.9</v>
       </c>
       <c r="L7" t="s">
         <v>15</v>
@@ -728,10 +728,10 @@
         <v>864997</v>
       </c>
       <c r="J8">
-        <v>20750000</v>
+        <v>248418378</v>
       </c>
       <c r="K8">
-        <v>4168.66</v>
+        <v>348.2</v>
       </c>
       <c r="L8" t="s">
         <v>13</v>
@@ -766,10 +766,10 @@
         <v>692599</v>
       </c>
       <c r="J9">
-        <v>20750000</v>
+        <v>248418378</v>
       </c>
       <c r="K9">
-        <v>3337.83</v>
+        <v>278.8</v>
       </c>
       <c r="L9" t="s">
         <v>14</v>
@@ -804,10 +804,10 @@
         <v>464094</v>
       </c>
       <c r="J10">
-        <v>20750000</v>
+        <v>248418378</v>
       </c>
       <c r="K10">
-        <v>2236.6</v>
+        <v>186.82</v>
       </c>
       <c r="L10" t="s">
         <v>15</v>
@@ -842,10 +842,10 @@
         <v>468005</v>
       </c>
       <c r="J11">
-        <v>15940000</v>
+        <v>172872079</v>
       </c>
       <c r="K11">
-        <v>2936.04</v>
+        <v>270.72</v>
       </c>
       <c r="L11" t="s">
         <v>13</v>
@@ -880,10 +880,10 @@
         <v>356596</v>
       </c>
       <c r="J12">
-        <v>15940000</v>
+        <v>172872079</v>
       </c>
       <c r="K12">
-        <v>2237.11</v>
+        <v>206.28</v>
       </c>
       <c r="L12" t="s">
         <v>14</v>
@@ -918,10 +918,10 @@
         <v>228812</v>
       </c>
       <c r="J13">
-        <v>15940000</v>
+        <v>172872079</v>
       </c>
       <c r="K13">
-        <v>1435.46</v>
+        <v>132.36</v>
       </c>
       <c r="L13" t="s">
         <v>15</v>
@@ -977,28 +977,28 @@
         <v>3359</v>
       </c>
       <c r="C2">
-        <v>3613.21</v>
+        <v>137008.26</v>
       </c>
       <c r="D2">
-        <v>2312.26</v>
+        <v>60.98</v>
       </c>
       <c r="E2">
-        <v>1.5</v>
+        <v>55.1</v>
       </c>
       <c r="F2">
-        <v>1</v>
+        <v>39.5</v>
       </c>
       <c r="G2">
-        <v>0.7</v>
+        <v>28.3</v>
       </c>
       <c r="H2">
         <v>83.2</v>
       </c>
       <c r="I2">
-        <v>29.34</v>
+        <v>0.77</v>
       </c>
       <c r="J2">
-        <v>-20</v>
+        <v>81.09</v>
       </c>
     </row>
     <row r="3" spans="1:10">
@@ -1009,28 +1009,28 @@
         <v>1196</v>
       </c>
       <c r="C3">
-        <v>2499.05</v>
+        <v>24996.4</v>
       </c>
       <c r="D3">
-        <v>397.22</v>
+        <v>39.71</v>
       </c>
       <c r="E3">
-        <v>3</v>
+        <v>30.1</v>
       </c>
       <c r="F3">
-        <v>2.2</v>
+        <v>21.6</v>
       </c>
       <c r="G3">
-        <v>1.8</v>
+        <v>18.1</v>
       </c>
       <c r="H3">
         <v>37.7</v>
       </c>
       <c r="I3">
-        <v>32.61</v>
+        <v>3.26</v>
       </c>
       <c r="J3">
-        <v>-20</v>
+        <v>38.34</v>
       </c>
     </row>
     <row r="4" spans="1:10">
@@ -1041,28 +1041,28 @@
         <v>661.5</v>
       </c>
       <c r="C4">
-        <v>1372.61</v>
+        <v>16432.88</v>
       </c>
       <c r="D4">
-        <v>267.47</v>
+        <v>22.34</v>
       </c>
       <c r="E4">
-        <v>2.5</v>
+        <v>29.6</v>
       </c>
       <c r="F4">
-        <v>1.7</v>
+        <v>20.3</v>
       </c>
       <c r="G4">
-        <v>1.1</v>
+        <v>12.6</v>
       </c>
       <c r="H4">
         <v>37.5</v>
       </c>
       <c r="I4">
-        <v>36.79</v>
+        <v>3.07</v>
       </c>
       <c r="J4">
-        <v>-20</v>
+        <v>34.92</v>
       </c>
     </row>
     <row r="5" spans="1:10">
@@ -1073,28 +1073,28 @@
         <v>829</v>
       </c>
       <c r="C5">
-        <v>1321.43</v>
+        <v>14331.1</v>
       </c>
       <c r="D5">
-        <v>138.02</v>
+        <v>12.73</v>
       </c>
       <c r="E5">
-        <v>6</v>
+        <v>65.09999999999999</v>
       </c>
       <c r="F5">
-        <v>3.8</v>
+        <v>40.9</v>
       </c>
       <c r="G5">
-        <v>1.9</v>
+        <v>20.2</v>
       </c>
       <c r="H5">
         <v>23.2</v>
       </c>
       <c r="I5">
-        <v>18.92</v>
+        <v>1.74</v>
       </c>
       <c r="J5">
-        <v>-11.78</v>
+        <v>52.8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>